<commit_message>
Updated 'GetTransactionData' WorkFlow and Added GetNextItem WorkFlow
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\TreasuryConfirmation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A33ABB6-F98E-4462-BB6B-C6A5F3C36194}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53296D95-6D83-4279-9154-89322B01904B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="334">
   <si>
     <t>Name</t>
   </si>
@@ -1021,6 +1021,12 @@
   </si>
   <si>
     <t>Treasury Confirmation - Error Occurred</t>
+  </si>
+  <si>
+    <t>MaxNumOfValidationLoops</t>
+  </si>
+  <si>
+    <t>Number</t>
   </si>
 </sst>
 </file>
@@ -2437,7 +2443,17 @@
       </c>
     </row>
     <row r="143" spans="1:3" ht="14" customHeight="1"/>
-    <row r="144" spans="1:3" ht="14" customHeight="1"/>
+    <row r="144" spans="1:3" ht="14" customHeight="1">
+      <c r="A144" t="s">
+        <v>332</v>
+      </c>
+      <c r="B144">
+        <v>3</v>
+      </c>
+      <c r="C144" t="s">
+        <v>333</v>
+      </c>
+    </row>
     <row r="145" spans="2:2" ht="14" customHeight="1"/>
     <row r="146" spans="2:2" ht="14" customHeight="1"/>
     <row r="147" spans="2:2" ht="14" customHeight="1"/>

</xml_diff>

<commit_message>
Updated 'ViewLogs' WorkFlow and Published 1.0.2 Package
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\TreasuryConfirmation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8F2822-7ACF-42AE-9988-536733FF8DC1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A155A14F-89C7-4751-A016-DB8FFA8E001F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="271">
   <si>
     <t>Name</t>
   </si>
@@ -722,9 +722,6 @@
     <t>Log_LogErrorMessage</t>
   </si>
   <si>
-    <t>Log Error Message -</t>
-  </si>
-  <si>
     <t>Log_ConfirmationEntry</t>
   </si>
   <si>
@@ -788,15 +785,9 @@
     <t>Log_ViewLogsEntry</t>
   </si>
   <si>
-    <t>Extracting Error Logs</t>
-  </si>
-  <si>
     <t>Log_ViewLogsEntrySuccess</t>
   </si>
   <si>
-    <t>Extracting Error Logs - Success</t>
-  </si>
-  <si>
     <t>Log_SingleRangeEntrySuccess</t>
   </si>
   <si>
@@ -824,13 +815,28 @@
     <t>Payment Instruction Fields did not match</t>
   </si>
   <si>
-    <t>ViewLogMatchPattern</t>
-  </si>
-  <si>
-    <t>(?:Error in)+(.+)</t>
-  </si>
-  <si>
     <t>TimeOut_BackOutRequestNumberNote</t>
+  </si>
+  <si>
+    <t>ViewLog_StartIndex</t>
+  </si>
+  <si>
+    <t>ViewLog_EndIndex</t>
+  </si>
+  <si>
+    <t>Start of log messages from FND_FILE</t>
+  </si>
+  <si>
+    <t>End of log messages from FND_FILE</t>
+  </si>
+  <si>
+    <t>Log Message(s) for Unconfirmed Payment Instruction -</t>
+  </si>
+  <si>
+    <t>Extracting Log Message(s) for Unconfirmed Payment Instruction</t>
+  </si>
+  <si>
+    <t>Extracting Log Message(s) for Unconfirmed Payment Instruction - Success</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1086"/>
+  <dimension ref="A1:Z1084"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -1660,7 +1666,7 @@
         <v>125</v>
       </c>
       <c r="B62" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.25" customHeight="1">
@@ -1700,119 +1706,119 @@
         <v>231</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>232</v>
+        <v>268</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="14.5">
       <c r="A68" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.5">
       <c r="A69" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.5">
       <c r="A70" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.5">
       <c r="A71" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.5">
       <c r="A73" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.5">
       <c r="A74" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.5">
       <c r="A75" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.5">
       <c r="A76" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="14.5">
       <c r="A77" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="14.5">
       <c r="A78" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="14.5">
       <c r="A79" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="14.5">
       <c r="A80" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="14.5">
       <c r="A81" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="14.5">
@@ -2432,61 +2438,65 @@
     </row>
     <row r="169" spans="1:3" ht="14.25" customHeight="1">
       <c r="A169" t="s">
+        <v>259</v>
+      </c>
+      <c r="B169" t="s">
         <v>262</v>
-      </c>
-      <c r="B169" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="170" spans="1:3" ht="14.25" customHeight="1">
       <c r="A170" t="s">
+        <v>260</v>
+      </c>
+      <c r="B170" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="172" spans="1:3" ht="15" customHeight="1">
+      <c r="A172" t="s">
         <v>263</v>
       </c>
-      <c r="B170" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="172" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A172" t="s">
-        <v>266</v>
-      </c>
-      <c r="B172" t="s">
-        <v>267</v>
+      <c r="B172">
+        <v>2</v>
+      </c>
+      <c r="C172" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="174" spans="1:3" ht="15" customHeight="1">
       <c r="A174" t="s">
-        <v>268</v>
-      </c>
-      <c r="B174">
-        <v>2</v>
-      </c>
-      <c r="C174" t="s">
-        <v>72</v>
+        <v>264</v>
+      </c>
+      <c r="B174" s="12" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" ht="15" customHeight="1">
+      <c r="A175" t="s">
+        <v>265</v>
+      </c>
+      <c r="B175" s="12" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="176" spans="1:3" ht="15" customHeight="1">
       <c r="B176" s="12"/>
     </row>
-    <row r="177" spans="2:2" ht="15" customHeight="1">
-      <c r="B177" s="12"/>
+    <row r="177" spans="2:2" ht="14.25" customHeight="1">
+      <c r="B177" s="2"/>
     </row>
     <row r="178" spans="2:2" ht="15" customHeight="1">
-      <c r="B178" s="12"/>
+      <c r="B178" s="2"/>
     </row>
     <row r="179" spans="2:2" ht="14.25" customHeight="1">
       <c r="B179" s="2"/>
     </row>
-    <row r="180" spans="2:2" ht="15" customHeight="1">
+    <row r="180" spans="2:2" ht="14.25" customHeight="1">
       <c r="B180" s="2"/>
     </row>
-    <row r="181" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B181" s="2"/>
-    </row>
-    <row r="182" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B182" s="2"/>
-    </row>
+    <row r="181" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="182" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="183" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="184" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="185" spans="2:2" ht="14.25" customHeight="1"/>
@@ -2509,29 +2519,37 @@
     <row r="202" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="203" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="204" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="205" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="206" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="205" spans="2:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="206" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B206" s="7"/>
+    </row>
+    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B207" s="7"/>
+    </row>
     <row r="208" spans="2:2" s="6" customFormat="1" ht="14.5">
       <c r="B208" s="7"/>
     </row>
-    <row r="209" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B209" s="7"/>
-    </row>
+    <row r="209" spans="1:3" s="6" customFormat="1" ht="14.5"/>
     <row r="210" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B210" s="7"/>
     </row>
-    <row r="211" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="211" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B211" s="7"/>
+    </row>
     <row r="212" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B212" s="7"/>
     </row>
-    <row r="213" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B213" s="7"/>
-    </row>
-    <row r="214" spans="1:3" s="6" customFormat="1" ht="14.5">
+    <row r="213" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="214" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A214" s="6"/>
       <c r="B214" s="7"/>
-    </row>
-    <row r="215" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="C214" s="6"/>
+    </row>
+    <row r="215" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A215" s="6"/>
+      <c r="B215" s="8"/>
+      <c r="C215" s="6"/>
+    </row>
     <row r="216" spans="1:3" ht="14.25" customHeight="1">
       <c r="A216" s="6"/>
       <c r="B216" s="7"/>
@@ -2539,58 +2557,50 @@
     </row>
     <row r="217" spans="1:3" ht="14.25" customHeight="1">
       <c r="A217" s="6"/>
-      <c r="B217" s="8"/>
+      <c r="B217" s="6"/>
       <c r="C217" s="6"/>
     </row>
     <row r="218" spans="1:3" ht="14.25" customHeight="1">
       <c r="A218" s="6"/>
-      <c r="B218" s="7"/>
+      <c r="B218" s="5"/>
       <c r="C218" s="6"/>
     </row>
     <row r="219" spans="1:3" ht="14.25" customHeight="1">
       <c r="A219" s="6"/>
-      <c r="B219" s="6"/>
+      <c r="B219" s="7"/>
       <c r="C219" s="6"/>
     </row>
     <row r="220" spans="1:3" ht="14.25" customHeight="1">
       <c r="A220" s="6"/>
-      <c r="B220" s="5"/>
+      <c r="B220" s="8"/>
       <c r="C220" s="6"/>
     </row>
     <row r="221" spans="1:3" ht="14.25" customHeight="1">
       <c r="A221" s="6"/>
-      <c r="B221" s="7"/>
+      <c r="B221" s="6"/>
       <c r="C221" s="6"/>
     </row>
     <row r="222" spans="1:3" ht="14.25" customHeight="1">
       <c r="A222" s="6"/>
-      <c r="B222" s="8"/>
+      <c r="B222" s="7"/>
       <c r="C222" s="6"/>
     </row>
-    <row r="223" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A223" s="6"/>
-      <c r="B223" s="6"/>
-      <c r="C223" s="6"/>
-    </row>
+    <row r="223" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="224" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A224" s="6"/>
-      <c r="B224" s="7"/>
-      <c r="C224" s="6"/>
-    </row>
-    <row r="225" spans="1:2" ht="14.25" customHeight="1"/>
+      <c r="B224" s="5"/>
+    </row>
+    <row r="225" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B225" s="7"/>
+    </row>
     <row r="226" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B226" s="5"/>
-    </row>
-    <row r="227" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B227" s="7"/>
-    </row>
+      <c r="B226" s="8"/>
+    </row>
+    <row r="227" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="228" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B228" s="8"/>
+      <c r="A228" s="6"/>
     </row>
     <row r="229" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="230" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A230" s="6"/>
-    </row>
+    <row r="230" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="231" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="232" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="233" spans="1:2" ht="14.25" customHeight="1"/>
@@ -3445,8 +3455,6 @@
     <row r="1082" ht="14.25" customHeight="1"/>
     <row r="1083" ht="14.25" customHeight="1"/>
     <row r="1084" ht="14.25" customHeight="1"/>
-    <row r="1085" ht="14.25" customHeight="1"/>
-    <row r="1086" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Upadated 'Config' File and Published New Package 1.0.5
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\TreasuryConfirmation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A155A14F-89C7-4751-A016-DB8FFA8E001F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D024997-91F8-436A-989C-C955D6980B6C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -310,9 +310,6 @@
     <t>Log_LaunchBrowser</t>
   </si>
   <si>
-    <t>PayablesManager</t>
-  </si>
-  <si>
     <t>SE_ErrMsg_NoEmptyBotStatusRowsFound</t>
   </si>
   <si>
@@ -837,6 +834,9 @@
   </si>
   <si>
     <t>Extracting Log Message(s) for Unconfirmed Payment Instruction - Success</t>
+  </si>
+  <si>
+    <t>TreasuryConfirmation</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1084"/>
+  <dimension ref="A1:Z1076"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -1280,7 +1280,7 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1330,7 +1330,7 @@
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>42</v>
@@ -1342,10 +1342,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B12" t="s">
         <v>155</v>
-      </c>
-      <c r="B12" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
@@ -1368,139 +1368,139 @@
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.5">
       <c r="A23" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5">
       <c r="A24" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.5">
       <c r="A26" t="s">
+        <v>206</v>
+      </c>
+      <c r="B26" t="s">
         <v>207</v>
-      </c>
-      <c r="B26" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15" customHeight="1">
       <c r="A27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B27" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5">
       <c r="A28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B28" t="s">
         <v>166</v>
-      </c>
-      <c r="B28" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.5">
       <c r="A29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B29" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.5">
       <c r="A30" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.5">
       <c r="A31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B31" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" t="s">
         <v>130</v>
-      </c>
-      <c r="B33" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
@@ -1508,7 +1508,7 @@
         <v>67</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1517,7 +1517,7 @@
         <v>49</v>
       </c>
       <c r="B36" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
@@ -1525,529 +1525,575 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="39" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="40" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="41" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="42" spans="1:2" ht="15" customHeight="1">
-      <c r="A42" t="s">
+    <row r="39" spans="1:2" ht="15" customHeight="1">
+      <c r="A39" t="s">
         <v>63</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B39" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="15" customHeight="1">
-      <c r="A43" t="s">
+    <row r="40" spans="1:2" ht="15" customHeight="1">
+      <c r="A40" t="s">
         <v>64</v>
       </c>
-      <c r="B43" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="15" customHeight="1">
+      <c r="B40" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15" customHeight="1">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A43" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="14.5">
       <c r="A44" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-    </row>
-    <row r="49" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A49" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>87</v>
+        <v>158</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="14.5">
+      <c r="A45" t="s">
+        <v>181</v>
+      </c>
+      <c r="B45" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.5">
+      <c r="A46" t="s">
+        <v>179</v>
+      </c>
+      <c r="B46" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="14.5">
+      <c r="A47" t="s">
+        <v>183</v>
+      </c>
+      <c r="B47" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="14.5">
+      <c r="A48" t="s">
+        <v>185</v>
+      </c>
+      <c r="B48" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="14.5">
+      <c r="A49" t="s">
+        <v>146</v>
+      </c>
+      <c r="B49" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.5">
       <c r="A50" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B50" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.5">
       <c r="A51" t="s">
-        <v>182</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
-        <v>183</v>
+        <v>93</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.5">
       <c r="A52" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="B52" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.5">
       <c r="A53" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B53" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.5">
       <c r="A54" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B54" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="14.5">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>147</v>
+        <v>123</v>
       </c>
       <c r="B55" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="14.5">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="B56" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="14.5">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>94</v>
+        <v>221</v>
       </c>
       <c r="B57" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="14.5">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>151</v>
+        <v>224</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>225</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.5">
-      <c r="A59" t="s">
-        <v>190</v>
-      </c>
-      <c r="B59" t="s">
-        <v>191</v>
+      <c r="A59" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.5">
-      <c r="A60" t="s">
-        <v>192</v>
-      </c>
-      <c r="B60" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A61" t="s">
-        <v>124</v>
-      </c>
-      <c r="B61" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A62" t="s">
-        <v>125</v>
-      </c>
-      <c r="B62" t="s">
+      <c r="A60" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="14.5">
+      <c r="A61" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="14.5">
+      <c r="A62" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="14.5">
+      <c r="A63" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A63" t="s">
-        <v>222</v>
-      </c>
-      <c r="B63" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A64" t="s">
-        <v>225</v>
-      </c>
-      <c r="B64" t="s">
-        <v>226</v>
+    <row r="64" spans="1:2" ht="14.5">
+      <c r="A64" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="14.5">
       <c r="A65" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.5">
       <c r="A66" s="2" t="s">
-        <v>129</v>
+        <v>237</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.5">
       <c r="A67" s="2" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="14.5">
       <c r="A68" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.5">
       <c r="A69" s="2" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.5">
       <c r="A70" s="2" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.5">
       <c r="A71" s="2" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.5">
       <c r="A73" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.5">
       <c r="A74" s="2" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.5">
       <c r="A75" s="2" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.5">
-      <c r="A76" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" ht="14.5">
-      <c r="A77" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="14.5">
-      <c r="A78" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="14.5">
-      <c r="A79" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="14.5">
-      <c r="A80" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="14.5">
-      <c r="A81" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="14.5">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-    </row>
-    <row r="83" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A83" t="s">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+    </row>
+    <row r="77" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A77" t="s">
         <v>88</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B77" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A84" t="s">
+    <row r="78" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A78" t="s">
+        <v>95</v>
+      </c>
+      <c r="B78" t="s">
         <v>96</v>
       </c>
-      <c r="B84" t="s">
+    </row>
+    <row r="79" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A79" t="s">
+        <v>89</v>
+      </c>
+      <c r="B79" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A80" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A81" t="s">
+        <v>108</v>
+      </c>
+      <c r="B81" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A83" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B83" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A84" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B84" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A85" s="2"/>
+      <c r="B85" s="2"/>
+    </row>
+    <row r="86" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A86" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B86" s="7">
+        <v>2000</v>
+      </c>
+      <c r="C86" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A87" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A88" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B88" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C88" s="6"/>
+    </row>
+    <row r="89" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A89" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B89" s="7">
+        <v>3</v>
+      </c>
+      <c r="C89" s="6"/>
+    </row>
+    <row r="90" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A90" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B90" s="7">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" ht="14.5"/>
+    <row r="92" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A92" t="s">
+        <v>91</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="94" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A94" t="s">
+        <v>109</v>
+      </c>
+      <c r="B94" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A95" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A85" t="s">
-        <v>89</v>
-      </c>
-      <c r="B85" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A86" t="s">
-        <v>105</v>
-      </c>
-      <c r="B86" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A87" t="s">
-        <v>109</v>
-      </c>
-      <c r="B87" t="s">
+      <c r="B95" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="97" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A97" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A88" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B88" s="2" t="s">
+      <c r="B97" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="89" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A89" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="B89" s="9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A90" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="B90" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-    </row>
-    <row r="92" spans="1:3" ht="15" customHeight="1">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-    </row>
-    <row r="93" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A93" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B93" s="7">
-        <v>2000</v>
-      </c>
-      <c r="C93" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A94" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B94">
-        <v>1</v>
-      </c>
-      <c r="C94" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A95" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B95" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C95" s="6"/>
-    </row>
-    <row r="96" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A96" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B96" s="7">
-        <v>3</v>
-      </c>
-      <c r="C96" s="6"/>
-    </row>
-    <row r="97" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A97" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B97" s="7">
-        <v>3</v>
-      </c>
-      <c r="C97" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" ht="14.5"/>
+    <row r="98" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A98" t="s">
+        <v>117</v>
+      </c>
+      <c r="B98" t="s">
+        <v>119</v>
+      </c>
+    </row>
     <row r="99" spans="1:3" ht="14.25" customHeight="1">
       <c r="A99" t="s">
-        <v>91</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="101" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A101" t="s">
-        <v>110</v>
-      </c>
-      <c r="B101" t="s">
-        <v>99</v>
-      </c>
-    </row>
+        <v>112</v>
+      </c>
+      <c r="B99" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A100" t="s">
+        <v>118</v>
+      </c>
+      <c r="B100" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="102" spans="1:3" ht="14.25" customHeight="1">
       <c r="A102" t="s">
-        <v>98</v>
-      </c>
-      <c r="B102" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>115</v>
+      </c>
+      <c r="B102">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A103" t="s">
+        <v>116</v>
+      </c>
+      <c r="B103">
+        <v>40000</v>
+      </c>
+      <c r="C103" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="104" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A104" t="s">
-        <v>112</v>
-      </c>
-      <c r="B104" t="s">
-        <v>115</v>
-      </c>
+      <c r="A104" s="6"/>
+      <c r="B104" s="7"/>
     </row>
     <row r="105" spans="1:3" ht="14.25" customHeight="1">
       <c r="A105" t="s">
-        <v>118</v>
-      </c>
-      <c r="B105" t="s">
-        <v>120</v>
+        <v>106</v>
+      </c>
+      <c r="B105">
+        <v>30000</v>
+      </c>
+      <c r="C105" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="106" spans="1:3" ht="14.25" customHeight="1">
       <c r="A106" t="s">
-        <v>113</v>
-      </c>
-      <c r="B106" t="s">
-        <v>114</v>
+        <v>103</v>
+      </c>
+      <c r="B106">
+        <v>30000</v>
+      </c>
+      <c r="C106" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="14.25" customHeight="1">
       <c r="A107" t="s">
-        <v>119</v>
-      </c>
-      <c r="B107" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>107</v>
+      </c>
+      <c r="B107">
+        <v>60000</v>
+      </c>
+      <c r="C107" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A108" s="6"/>
+      <c r="B108" s="7"/>
+      <c r="C108" s="6"/>
+    </row>
     <row r="109" spans="1:3" ht="14.25" customHeight="1">
       <c r="A109" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="B109">
-        <v>2</v>
+        <v>2000</v>
+      </c>
+      <c r="C109" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="110" spans="1:3" ht="14.25" customHeight="1">
       <c r="A110" t="s">
-        <v>117</v>
+        <v>76</v>
       </c>
       <c r="B110">
-        <v>40000</v>
-      </c>
-      <c r="C110" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A111" s="6"/>
-      <c r="B111" s="7"/>
-    </row>
-    <row r="112" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A112" t="s">
-        <v>107</v>
-      </c>
-      <c r="B112">
-        <v>30000</v>
-      </c>
-      <c r="C112" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A111" t="s">
+        <v>77</v>
+      </c>
+      <c r="B111">
+        <v>1</v>
+      </c>
+      <c r="C111" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="113" spans="1:3" ht="15" customHeight="1">
       <c r="A113" t="s">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="B113">
-        <v>30000</v>
+        <v>2000</v>
       </c>
       <c r="C113" t="s">
         <v>72</v>
@@ -2055,562 +2101,511 @@
     </row>
     <row r="114" spans="1:3" ht="14.25" customHeight="1">
       <c r="A114" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="B114">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A115" t="s">
+        <v>79</v>
+      </c>
+      <c r="B115">
+        <v>1</v>
+      </c>
+      <c r="C115" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" ht="17.5" customHeight="1"/>
+    <row r="117" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A117" t="s">
+        <v>152</v>
+      </c>
+      <c r="B117">
+        <v>3000</v>
+      </c>
+      <c r="C117" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="119" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A119" t="s">
+        <v>121</v>
+      </c>
+      <c r="B119" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A120" s="6"/>
+      <c r="B120" s="7"/>
+      <c r="C120" s="6"/>
+    </row>
+    <row r="121" spans="1:3" ht="14" customHeight="1">
+      <c r="A121" t="s">
+        <v>122</v>
+      </c>
+      <c r="B121">
+        <v>1</v>
+      </c>
+      <c r="C121" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="123" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A123" t="s">
+        <v>134</v>
+      </c>
+      <c r="B123">
         <v>60000</v>
       </c>
-      <c r="C114" t="s">
+      <c r="C123" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="115" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A115" s="6"/>
-      <c r="B115" s="7"/>
-      <c r="C115" s="6"/>
-    </row>
-    <row r="116" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A116" t="s">
-        <v>74</v>
-      </c>
-      <c r="B116">
-        <v>2000</v>
-      </c>
-      <c r="C116" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A117" t="s">
-        <v>76</v>
-      </c>
-      <c r="B117">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A118" t="s">
-        <v>77</v>
-      </c>
-      <c r="B118">
-        <v>1</v>
-      </c>
-      <c r="C118" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="120" spans="1:3" ht="15" customHeight="1">
-      <c r="A120" t="s">
-        <v>75</v>
-      </c>
-      <c r="B120">
-        <v>2000</v>
-      </c>
-      <c r="C120" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A121" t="s">
-        <v>78</v>
-      </c>
-      <c r="B121">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A122" t="s">
-        <v>79</v>
-      </c>
-      <c r="B122">
-        <v>1</v>
-      </c>
-      <c r="C122" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="124" spans="1:3" ht="17.5" customHeight="1">
+    <row r="124" spans="1:3" ht="14.25" customHeight="1">
       <c r="A124" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
       <c r="B124">
-        <v>3000</v>
+        <v>60000</v>
       </c>
       <c r="C124" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="125" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="126" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A126" t="s">
-        <v>122</v>
-      </c>
-      <c r="B126" t="s">
-        <v>189</v>
-      </c>
-    </row>
+    <row r="125" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A125" t="s">
+        <v>135</v>
+      </c>
+      <c r="B125">
+        <v>60000</v>
+      </c>
+      <c r="C125" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="127" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A127" s="6"/>
-      <c r="B127" s="7"/>
-      <c r="C127" s="6"/>
-    </row>
-    <row r="128" spans="1:3" ht="14" customHeight="1">
-      <c r="A128" t="s">
-        <v>123</v>
-      </c>
-      <c r="B128">
-        <v>1</v>
-      </c>
-      <c r="C128" t="s">
+      <c r="A127" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="B127" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" ht="17.5" customHeight="1"/>
+    <row r="129" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A129" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B129" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A130" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B130" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A131" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A132" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B132" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="134" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A134" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B134" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A135" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A136" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B136" s="7">
+        <v>60</v>
+      </c>
+      <c r="C136" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="130" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A130" t="s">
-        <v>135</v>
-      </c>
-      <c r="B130">
-        <v>60000</v>
-      </c>
-      <c r="C130" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A131" t="s">
-        <v>134</v>
-      </c>
-      <c r="B131">
-        <v>60000</v>
-      </c>
-      <c r="C131" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A132" t="s">
+    <row r="137" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="138" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A138" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B138" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C138" s="6"/>
+    </row>
+    <row r="139" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A139" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C139" s="6"/>
+    </row>
+    <row r="140" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A140" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B140" s="7">
+        <v>60</v>
+      </c>
+      <c r="C140" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A141" s="6"/>
+      <c r="B141" s="6"/>
+      <c r="C141" s="6"/>
+    </row>
+    <row r="142" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A142" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="B132">
-        <v>60000</v>
-      </c>
-      <c r="C132" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="134" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A134" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B134" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="136" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="137" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A137" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B137" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A138" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B138" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A139" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B139" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A140" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B140" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="142" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A142" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B142" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B142" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C142" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="14.25" customHeight="1">
       <c r="A143" s="6" t="s">
-        <v>59</v>
+        <v>137</v>
       </c>
       <c r="B143" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" s="6" customFormat="1" ht="14.5">
+        <v>208</v>
+      </c>
+      <c r="C143" s="6"/>
+    </row>
+    <row r="144" spans="1:3" ht="14.25" customHeight="1">
       <c r="A144" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B144" s="7">
-        <v>60</v>
-      </c>
-      <c r="C144" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>138</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C144" s="6"/>
+    </row>
+    <row r="145" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A145" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B145" s="6"/>
+      <c r="C145" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="146" spans="1:3" ht="14.25" customHeight="1">
       <c r="A146" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B146" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C146" s="6"/>
-    </row>
-    <row r="147" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A147" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B147" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C147" s="6"/>
-    </row>
+        <v>47</v>
+      </c>
+      <c r="B146" s="7">
+        <v>60000</v>
+      </c>
+      <c r="C146" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="148" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A148" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B148" s="7">
-        <v>60</v>
-      </c>
-      <c r="C148" s="6" t="s">
-        <v>61</v>
+      <c r="A148" t="s">
+        <v>139</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="149" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A149" s="6"/>
-      <c r="B149" s="6"/>
-      <c r="C149" s="6"/>
+      <c r="A149" t="s">
+        <v>140</v>
+      </c>
+      <c r="B149" s="7" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="150" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A150" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C150" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A151" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B151" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="C151" s="6"/>
-    </row>
-    <row r="152" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A152" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="B152" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="C152" s="6"/>
-    </row>
-    <row r="153" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A153" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B153" s="6"/>
-      <c r="C153" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A154" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B154" s="7">
-        <v>60000</v>
-      </c>
-      <c r="C154" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="156" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A150" t="s">
+        <v>141</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" ht="14" customHeight="1"/>
+    <row r="152" spans="1:3" ht="14" customHeight="1">
+      <c r="A152" t="s">
+        <v>211</v>
+      </c>
+      <c r="B152">
+        <v>3</v>
+      </c>
+      <c r="C152" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" ht="14" customHeight="1"/>
+    <row r="154" spans="1:3" ht="14" customHeight="1">
+      <c r="A154" t="s">
+        <v>213</v>
+      </c>
+      <c r="B154" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" ht="14" customHeight="1"/>
+    <row r="156" spans="1:3" ht="14" customHeight="1">
       <c r="A156" t="s">
-        <v>140</v>
-      </c>
-      <c r="B156" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" ht="14.25" customHeight="1">
+        <v>217</v>
+      </c>
+      <c r="B156" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" ht="14" customHeight="1">
       <c r="A157" t="s">
-        <v>141</v>
-      </c>
-      <c r="B157" s="7" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A158" t="s">
-        <v>142</v>
-      </c>
-      <c r="B158" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" ht="14" customHeight="1"/>
-    <row r="160" spans="1:3" ht="14" customHeight="1">
+        <v>218</v>
+      </c>
+      <c r="B157" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" ht="14" customHeight="1"/>
+    <row r="159" spans="1:3" ht="15" customHeight="1">
+      <c r="A159" t="s">
+        <v>219</v>
+      </c>
+      <c r="B159" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" ht="14.25" customHeight="1">
       <c r="A160" t="s">
-        <v>212</v>
-      </c>
-      <c r="B160">
-        <v>3</v>
-      </c>
-      <c r="C160" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" ht="14" customHeight="1"/>
-    <row r="162" spans="1:3" ht="14" customHeight="1">
+        <v>223</v>
+      </c>
+      <c r="B160" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A161" t="s">
+        <v>258</v>
+      </c>
+      <c r="B161" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" ht="14.25" customHeight="1">
       <c r="A162" t="s">
-        <v>214</v>
+        <v>259</v>
       </c>
       <c r="B162" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="14" customHeight="1"/>
-    <row r="164" spans="1:3" ht="14" customHeight="1">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="164" spans="1:3" ht="15" customHeight="1">
       <c r="A164" t="s">
-        <v>218</v>
-      </c>
-      <c r="B164" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="14" customHeight="1">
-      <c r="A165" t="s">
-        <v>219</v>
-      </c>
-      <c r="B165" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" ht="14" customHeight="1"/>
+        <v>262</v>
+      </c>
+      <c r="B164">
+        <v>2</v>
+      </c>
+      <c r="C164" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" ht="15" customHeight="1">
+      <c r="A166" t="s">
+        <v>263</v>
+      </c>
+      <c r="B166" s="12" t="s">
+        <v>265</v>
+      </c>
+    </row>
     <row r="167" spans="1:3" ht="15" customHeight="1">
       <c r="A167" t="s">
-        <v>220</v>
+        <v>264</v>
       </c>
       <c r="B167" s="12" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A168" t="s">
-        <v>224</v>
-      </c>
-      <c r="B168" t="s">
-        <v>223</v>
-      </c>
+        <v>266</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="15" customHeight="1">
+      <c r="B168" s="12"/>
     </row>
     <row r="169" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A169" t="s">
-        <v>259</v>
-      </c>
-      <c r="B169" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A170" t="s">
-        <v>260</v>
-      </c>
-      <c r="B170" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="172" spans="1:3" ht="15" customHeight="1">
-      <c r="A172" t="s">
-        <v>263</v>
-      </c>
-      <c r="B172">
-        <v>2</v>
-      </c>
-      <c r="C172" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" ht="15" customHeight="1">
-      <c r="A174" t="s">
-        <v>264</v>
-      </c>
-      <c r="B174" s="12" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" ht="15" customHeight="1">
-      <c r="A175" t="s">
-        <v>265</v>
-      </c>
-      <c r="B175" s="12" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" ht="15" customHeight="1">
-      <c r="B176" s="12"/>
-    </row>
-    <row r="177" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B177" s="2"/>
-    </row>
-    <row r="178" spans="2:2" ht="15" customHeight="1">
-      <c r="B178" s="2"/>
-    </row>
-    <row r="179" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B179" s="2"/>
-    </row>
-    <row r="180" spans="2:2" ht="14.25" customHeight="1">
-      <c r="B180" s="2"/>
-    </row>
-    <row r="181" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="182" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="183" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="184" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="185" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="186" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="187" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="188" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="189" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="190" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="191" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="192" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="193" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="194" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="195" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="196" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="197" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="198" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="199" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="200" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="201" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="202" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="203" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="204" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="205" spans="2:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="206" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B169" s="2"/>
+    </row>
+    <row r="170" spans="1:3" ht="15" customHeight="1">
+      <c r="B170" s="2"/>
+    </row>
+    <row r="171" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B171" s="2"/>
+    </row>
+    <row r="172" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B172" s="2"/>
+    </row>
+    <row r="173" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="174" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="175" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="176" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="177" ht="14.25" customHeight="1"/>
+    <row r="178" ht="14.25" customHeight="1"/>
+    <row r="179" ht="14.25" customHeight="1"/>
+    <row r="180" ht="14.25" customHeight="1"/>
+    <row r="181" ht="14.25" customHeight="1"/>
+    <row r="182" ht="14.25" customHeight="1"/>
+    <row r="183" ht="14.25" customHeight="1"/>
+    <row r="184" ht="14.25" customHeight="1"/>
+    <row r="185" ht="14.25" customHeight="1"/>
+    <row r="186" ht="14.25" customHeight="1"/>
+    <row r="187" ht="14.25" customHeight="1"/>
+    <row r="188" ht="14.25" customHeight="1"/>
+    <row r="189" ht="14.25" customHeight="1"/>
+    <row r="190" ht="14.25" customHeight="1"/>
+    <row r="191" ht="14.25" customHeight="1"/>
+    <row r="192" ht="14.25" customHeight="1"/>
+    <row r="193" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="194" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="195" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="196" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="197" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="198" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B198" s="7"/>
+    </row>
+    <row r="199" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B199" s="7"/>
+    </row>
+    <row r="200" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B200" s="7"/>
+    </row>
+    <row r="201" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="202" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B202" s="7"/>
+    </row>
+    <row r="203" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B203" s="7"/>
+    </row>
+    <row r="204" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B204" s="7"/>
+    </row>
+    <row r="205" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="206" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A206" s="6"/>
       <c r="B206" s="7"/>
-    </row>
-    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B207" s="7"/>
-    </row>
-    <row r="208" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="C206" s="6"/>
+    </row>
+    <row r="207" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A207" s="6"/>
+      <c r="B207" s="8"/>
+      <c r="C207" s="6"/>
+    </row>
+    <row r="208" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A208" s="6"/>
       <c r="B208" s="7"/>
-    </row>
-    <row r="209" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="210" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B210" s="7"/>
-    </row>
-    <row r="211" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="C208" s="6"/>
+    </row>
+    <row r="209" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A209" s="6"/>
+      <c r="B209" s="6"/>
+      <c r="C209" s="6"/>
+    </row>
+    <row r="210" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A210" s="6"/>
+      <c r="B210" s="5"/>
+      <c r="C210" s="6"/>
+    </row>
+    <row r="211" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A211" s="6"/>
       <c r="B211" s="7"/>
-    </row>
-    <row r="212" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B212" s="7"/>
-    </row>
-    <row r="213" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="C211" s="6"/>
+    </row>
+    <row r="212" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A212" s="6"/>
+      <c r="B212" s="8"/>
+      <c r="C212" s="6"/>
+    </row>
+    <row r="213" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A213" s="6"/>
+      <c r="B213" s="6"/>
+      <c r="C213" s="6"/>
+    </row>
     <row r="214" spans="1:3" ht="14.25" customHeight="1">
       <c r="A214" s="6"/>
       <c r="B214" s="7"/>
       <c r="C214" s="6"/>
     </row>
-    <row r="215" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A215" s="6"/>
-      <c r="B215" s="8"/>
-      <c r="C215" s="6"/>
-    </row>
+    <row r="215" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="216" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A216" s="6"/>
-      <c r="B216" s="7"/>
-      <c r="C216" s="6"/>
+      <c r="B216" s="5"/>
     </row>
     <row r="217" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A217" s="6"/>
-      <c r="B217" s="6"/>
-      <c r="C217" s="6"/>
+      <c r="B217" s="7"/>
     </row>
     <row r="218" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A218" s="6"/>
-      <c r="B218" s="5"/>
-      <c r="C218" s="6"/>
-    </row>
-    <row r="219" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A219" s="6"/>
-      <c r="B219" s="7"/>
-      <c r="C219" s="6"/>
-    </row>
+      <c r="B218" s="8"/>
+    </row>
+    <row r="219" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="220" spans="1:3" ht="14.25" customHeight="1">
       <c r="A220" s="6"/>
-      <c r="B220" s="8"/>
-      <c r="C220" s="6"/>
-    </row>
-    <row r="221" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A221" s="6"/>
-      <c r="B221" s="6"/>
-      <c r="C221" s="6"/>
-    </row>
-    <row r="222" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A222" s="6"/>
-      <c r="B222" s="7"/>
-      <c r="C222" s="6"/>
-    </row>
+    </row>
+    <row r="221" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="222" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="223" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="224" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B224" s="5"/>
-    </row>
-    <row r="225" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B225" s="7"/>
-    </row>
-    <row r="226" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B226" s="8"/>
-    </row>
-    <row r="227" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="228" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A228" s="6"/>
-    </row>
-    <row r="229" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="230" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="231" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="232" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="233" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="234" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="235" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="236" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="237" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="238" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="239" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="240" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="224" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="225" ht="14.25" customHeight="1"/>
+    <row r="226" ht="14.25" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
+    <row r="228" ht="14.25" customHeight="1"/>
+    <row r="229" ht="14.25" customHeight="1"/>
+    <row r="230" ht="14.25" customHeight="1"/>
+    <row r="231" ht="14.25" customHeight="1"/>
+    <row r="232" ht="14.25" customHeight="1"/>
+    <row r="233" ht="14.25" customHeight="1"/>
+    <row r="234" ht="14.25" customHeight="1"/>
+    <row r="235" ht="14.25" customHeight="1"/>
+    <row r="236" ht="14.25" customHeight="1"/>
+    <row r="237" ht="14.25" customHeight="1"/>
+    <row r="238" ht="14.25" customHeight="1"/>
+    <row r="239" ht="14.25" customHeight="1"/>
+    <row r="240" ht="14.25" customHeight="1"/>
     <row r="241" ht="14.25" customHeight="1"/>
     <row r="242" ht="14.25" customHeight="1"/>
     <row r="243" ht="14.25" customHeight="1"/>
@@ -3447,14 +3442,6 @@
     <row r="1074" ht="14.25" customHeight="1"/>
     <row r="1075" ht="14.25" customHeight="1"/>
     <row r="1076" ht="14.25" customHeight="1"/>
-    <row r="1077" ht="14.25" customHeight="1"/>
-    <row r="1078" ht="14.25" customHeight="1"/>
-    <row r="1079" ht="14.25" customHeight="1"/>
-    <row r="1080" ht="14.25" customHeight="1"/>
-    <row r="1081" ht="14.25" customHeight="1"/>
-    <row r="1082" ht="14.25" customHeight="1"/>
-    <row r="1083" ht="14.25" customHeight="1"/>
-    <row r="1084" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3649,7 +3636,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Added 'AdjustRowHeight' WorkFlow, Updated activities with Simulate and Send window messages properties
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\TreasuryConfirmation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D024997-91F8-436A-989C-C955D6980B6C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8C208C-0875-40D7-B243-E60BCF163E93}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="280">
   <si>
     <t>Name</t>
   </si>
@@ -455,9 +455,6 @@
 Error message is: </t>
   </si>
   <si>
-    <t>gmahesh2789@gmail.com; sunil.melam@gmail.com; hariharangouri@gmail.com</t>
-  </si>
-  <si>
     <t>Log_TransactionComplete</t>
   </si>
   <si>
@@ -837,6 +834,36 @@
   </si>
   <si>
     <t>TreasuryConfirmation</t>
+  </si>
+  <si>
+    <t>TimeOut_ErrorDisplayed</t>
+  </si>
+  <si>
+    <t>TimeOut_PaymentInstructionDropdownDisplayed</t>
+  </si>
+  <si>
+    <t>Status_Confirmed</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>Status_UnConfirmed</t>
+  </si>
+  <si>
+    <t>Unconfirmed</t>
+  </si>
+  <si>
+    <t>AdjustRowHeight</t>
+  </si>
+  <si>
+    <t>in number</t>
+  </si>
+  <si>
+    <t>gmahesh2789@gmail.com; hariharangouri@gmail.com</t>
+  </si>
+  <si>
+    <t>gmahesh2789@gmail.com; hariharangouri@gmail.com; sunil.melam@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1076"/>
+  <dimension ref="A1:Z1079"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -1280,7 +1307,7 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1330,7 +1357,7 @@
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>42</v>
@@ -1342,10 +1369,10 @@
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" t="s">
         <v>154</v>
-      </c>
-      <c r="B12" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
@@ -1376,122 +1403,122 @@
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.5">
       <c r="A23" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5">
       <c r="A24" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.5">
       <c r="A26" t="s">
+        <v>205</v>
+      </c>
+      <c r="B26" t="s">
         <v>206</v>
-      </c>
-      <c r="B26" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15" customHeight="1">
       <c r="A27" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5">
       <c r="A28" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" t="s">
         <v>165</v>
-      </c>
-      <c r="B28" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.5">
       <c r="A29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.5">
       <c r="A30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.5">
       <c r="A31" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1517,7 +1544,7 @@
         <v>49</v>
       </c>
       <c r="B36" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
@@ -1559,58 +1586,58 @@
     </row>
     <row r="44" spans="1:2" ht="14.5">
       <c r="A44" t="s">
+        <v>156</v>
+      </c>
+      <c r="B44" t="s">
         <v>157</v>
-      </c>
-      <c r="B44" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.5">
       <c r="A45" t="s">
+        <v>180</v>
+      </c>
+      <c r="B45" t="s">
         <v>181</v>
-      </c>
-      <c r="B45" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.5">
       <c r="A46" t="s">
+        <v>178</v>
+      </c>
+      <c r="B46" t="s">
         <v>179</v>
-      </c>
-      <c r="B46" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.5">
       <c r="A47" t="s">
+        <v>182</v>
+      </c>
+      <c r="B47" t="s">
         <v>183</v>
-      </c>
-      <c r="B47" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.5">
       <c r="A48" t="s">
+        <v>184</v>
+      </c>
+      <c r="B48" t="s">
         <v>185</v>
-      </c>
-      <c r="B48" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.5">
       <c r="A49" t="s">
+        <v>145</v>
+      </c>
+      <c r="B49" t="s">
         <v>146</v>
-      </c>
-      <c r="B49" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.5">
       <c r="A50" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50" t="s">
         <v>148</v>
-      </c>
-      <c r="B50" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.5">
@@ -1623,26 +1650,26 @@
     </row>
     <row r="52" spans="1:2" ht="14.5">
       <c r="A52" t="s">
+        <v>149</v>
+      </c>
+      <c r="B52" t="s">
         <v>150</v>
-      </c>
-      <c r="B52" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.5">
       <c r="A53" t="s">
+        <v>188</v>
+      </c>
+      <c r="B53" t="s">
         <v>189</v>
-      </c>
-      <c r="B53" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.5">
       <c r="A54" t="s">
+        <v>190</v>
+      </c>
+      <c r="B54" t="s">
         <v>191</v>
-      </c>
-      <c r="B54" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
@@ -1658,31 +1685,31 @@
         <v>124</v>
       </c>
       <c r="B56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B57" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.25" customHeight="1">
       <c r="A58" t="s">
+        <v>223</v>
+      </c>
+      <c r="B58" t="s">
         <v>224</v>
-      </c>
-      <c r="B58" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.5">
       <c r="A59" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.5">
@@ -1690,127 +1717,127 @@
         <v>128</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.5">
       <c r="A61" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="14.5">
       <c r="A62" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.5">
       <c r="A63" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.5">
       <c r="A64" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="14.5">
       <c r="A65" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.5">
       <c r="A66" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.5">
       <c r="A67" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="14.5">
       <c r="A68" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="14.5">
       <c r="A69" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.5">
       <c r="A70" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.5">
       <c r="A71" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.5">
       <c r="A73" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.5">
       <c r="A74" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.5">
       <c r="A75" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.5">
@@ -1859,7 +1886,7 @@
     </row>
     <row r="82" spans="1:3" ht="14.25" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>113</v>
@@ -1867,18 +1894,18 @@
     </row>
     <row r="83" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
       <c r="A83" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B83" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="B83" s="9" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="84" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
       <c r="A84" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B84" s="9" t="s">
         <v>193</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="14.25" customHeight="1">
@@ -2121,7 +2148,7 @@
     <row r="116" spans="1:3" ht="17.5" customHeight="1"/>
     <row r="117" spans="1:3" ht="17.5" customHeight="1">
       <c r="A117" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B117">
         <v>3000</v>
@@ -2136,7 +2163,7 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="14.25" customHeight="1">
@@ -2189,302 +2216,348 @@
         <v>72</v>
       </c>
     </row>
-    <row r="126" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="126" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A126" t="s">
+        <v>270</v>
+      </c>
+      <c r="B126">
+        <v>5</v>
+      </c>
+      <c r="C126" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="127" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A127" s="6" t="s">
+      <c r="A127" t="s">
+        <v>271</v>
+      </c>
+      <c r="B127">
+        <v>5</v>
+      </c>
+      <c r="C127" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" ht="14.5" customHeight="1">
+      <c r="A128" t="s">
+        <v>261</v>
+      </c>
+      <c r="B128">
+        <v>5</v>
+      </c>
+      <c r="C128" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="130" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A130" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B130" t="s">
         <v>144</v>
       </c>
-      <c r="B127" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="129" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A129" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B129" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A130" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B130" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A131" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B131" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
+    </row>
+    <row r="131" spans="1:3" ht="17.5" customHeight="1"/>
     <row r="132" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A132" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B132" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+        <v>50</v>
+      </c>
+      <c r="B132" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A133" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B133" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="134" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A134" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="135" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="A135" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="137" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A137" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A138" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B135" s="7" t="s">
+      <c r="B138" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="136" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A136" s="6" t="s">
+    <row r="139" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A139" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B136" s="7">
+      <c r="B139" s="7">
         <v>60</v>
       </c>
-      <c r="C136" s="6" t="s">
+      <c r="C139" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="137" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="138" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A138" s="6" t="s">
+    <row r="140" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="141" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A141" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B138" s="7" t="s">
+      <c r="B141" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C138" s="6"/>
-    </row>
-    <row r="139" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A139" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B139" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C139" s="6"/>
-    </row>
-    <row r="140" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A140" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B140" s="7">
-        <v>60</v>
-      </c>
-      <c r="C140" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A141" s="6"/>
-      <c r="B141" s="6"/>
       <c r="C141" s="6"/>
     </row>
     <row r="142" spans="1:3" ht="14.25" customHeight="1">
       <c r="A142" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="C142" s="6" t="s">
-        <v>45</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C142" s="6"/>
     </row>
     <row r="143" spans="1:3" ht="14.25" customHeight="1">
       <c r="A143" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B143" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="C143" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="B143" s="7">
+        <v>60</v>
+      </c>
+      <c r="C143" s="6" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="144" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A144" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B144" s="8" t="s">
-        <v>209</v>
-      </c>
+      <c r="A144" s="6"/>
+      <c r="B144" s="6"/>
       <c r="C144" s="6"/>
     </row>
     <row r="145" spans="1:3" ht="14.25" customHeight="1">
       <c r="A145" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B145" s="6"/>
+        <v>136</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>278</v>
+      </c>
       <c r="C145" s="6" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="146" spans="1:3" ht="14.25" customHeight="1">
       <c r="A146" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B146" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C146" s="6"/>
+    </row>
+    <row r="147" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A147" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C147" s="6"/>
+    </row>
+    <row r="148" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A148" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B148" s="6"/>
+      <c r="C148" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A149" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B146" s="7">
+      <c r="B149" s="7">
         <v>60000</v>
       </c>
-      <c r="C146" s="6" t="s">
+      <c r="C149" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="147" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="148" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A148" t="s">
+    <row r="150" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="151" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A151" t="s">
         <v>139</v>
       </c>
-      <c r="B148" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A149" t="s">
+      <c r="B151" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="C151" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A152" t="s">
         <v>140</v>
       </c>
-      <c r="B149" s="7" t="s">
+      <c r="B152" s="7" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A153" t="s">
+        <v>141</v>
+      </c>
+      <c r="B153" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" ht="14" customHeight="1"/>
+    <row r="155" spans="1:3" ht="14" customHeight="1">
+      <c r="A155" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="150" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A150" t="s">
-        <v>141</v>
-      </c>
-      <c r="B150" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" ht="14" customHeight="1"/>
-    <row r="152" spans="1:3" ht="14" customHeight="1">
-      <c r="A152" t="s">
+      <c r="B155">
+        <v>5</v>
+      </c>
+      <c r="C155" t="s">
         <v>211</v>
       </c>
-      <c r="B152">
-        <v>3</v>
-      </c>
-      <c r="C152" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" ht="14" customHeight="1"/>
-    <row r="154" spans="1:3" ht="14" customHeight="1">
-      <c r="A154" t="s">
-        <v>213</v>
-      </c>
-      <c r="B154" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" ht="14" customHeight="1"/>
-    <row r="156" spans="1:3" ht="14" customHeight="1">
-      <c r="A156" t="s">
-        <v>217</v>
-      </c>
-      <c r="B156" t="s">
-        <v>215</v>
-      </c>
-    </row>
+    </row>
+    <row r="156" spans="1:3" ht="14" customHeight="1"/>
     <row r="157" spans="1:3" ht="14" customHeight="1">
       <c r="A157" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B157" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" ht="14" customHeight="1">
+      <c r="A158" t="s">
+        <v>272</v>
+      </c>
+      <c r="B158" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" ht="14" customHeight="1">
+      <c r="A159" t="s">
+        <v>274</v>
+      </c>
+      <c r="B159" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" ht="14" customHeight="1"/>
+    <row r="161" spans="1:3" ht="14" customHeight="1">
+      <c r="A161" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="158" spans="1:3" ht="14" customHeight="1"/>
-    <row r="159" spans="1:3" ht="15" customHeight="1">
-      <c r="A159" t="s">
-        <v>219</v>
-      </c>
-      <c r="B159" s="12" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A160" t="s">
-        <v>223</v>
-      </c>
-      <c r="B160" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A161" t="s">
-        <v>258</v>
-      </c>
       <c r="B161" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" ht="14.25" customHeight="1">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" ht="14" customHeight="1">
       <c r="A162" t="s">
-        <v>259</v>
+        <v>217</v>
       </c>
       <c r="B162" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>215</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" ht="14" customHeight="1"/>
     <row r="164" spans="1:3" ht="15" customHeight="1">
       <c r="A164" t="s">
+        <v>218</v>
+      </c>
+      <c r="B164" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A165" t="s">
+        <v>222</v>
+      </c>
+      <c r="B165" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A166" t="s">
+        <v>257</v>
+      </c>
+      <c r="B166" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A167" t="s">
+        <v>258</v>
+      </c>
+      <c r="B167" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="169" spans="1:3" ht="15" customHeight="1">
+      <c r="A169" t="s">
         <v>262</v>
       </c>
-      <c r="B164">
-        <v>2</v>
-      </c>
-      <c r="C164" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" ht="15" customHeight="1">
-      <c r="A166" t="s">
+      <c r="B169" s="12" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" ht="15" customHeight="1">
+      <c r="A170" t="s">
         <v>263</v>
       </c>
-      <c r="B166" s="12" t="s">
+      <c r="B170" s="12" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="167" spans="1:3" ht="15" customHeight="1">
-      <c r="A167" t="s">
-        <v>264</v>
-      </c>
-      <c r="B167" s="12" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" ht="15" customHeight="1">
-      <c r="B168" s="12"/>
-    </row>
-    <row r="169" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B169" s="2"/>
-    </row>
-    <row r="170" spans="1:3" ht="15" customHeight="1">
-      <c r="B170" s="2"/>
-    </row>
-    <row r="171" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B171" s="2"/>
+    <row r="171" spans="1:3" ht="15" customHeight="1">
+      <c r="B171" s="12"/>
     </row>
     <row r="172" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B172" s="2"/>
-    </row>
-    <row r="173" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="174" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="175" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="A172" t="s">
+        <v>276</v>
+      </c>
+      <c r="B172" s="2">
+        <v>25</v>
+      </c>
+      <c r="C172" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" ht="15" customHeight="1">
+      <c r="B173" s="2"/>
+    </row>
+    <row r="174" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B174" s="2"/>
+    </row>
+    <row r="175" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B175" s="2"/>
+    </row>
     <row r="176" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="177" ht="14.25" customHeight="1"/>
     <row r="178" ht="14.25" customHeight="1"/>
@@ -2502,54 +2575,42 @@
     <row r="190" ht="14.25" customHeight="1"/>
     <row r="191" ht="14.25" customHeight="1"/>
     <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="194" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="195" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="196" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="197" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="198" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B198" s="7"/>
-    </row>
-    <row r="199" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B199" s="7"/>
-    </row>
-    <row r="200" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B200" s="7"/>
-    </row>
-    <row r="201" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="202" spans="1:3" s="6" customFormat="1" ht="14.5">
+    <row r="193" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="194" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="195" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="196" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="197" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="198" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="199" spans="2:2" ht="14.25" customHeight="1"/>
+    <row r="200" spans="2:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="201" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B201" s="7"/>
+    </row>
+    <row r="202" spans="2:2" s="6" customFormat="1" ht="14.5">
       <c r="B202" s="7"/>
     </row>
-    <row r="203" spans="1:3" s="6" customFormat="1" ht="14.5">
+    <row r="203" spans="2:2" s="6" customFormat="1" ht="14.5">
       <c r="B203" s="7"/>
     </row>
-    <row r="204" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B204" s="7"/>
-    </row>
-    <row r="205" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="206" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A206" s="6"/>
+    <row r="204" spans="2:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="205" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B205" s="7"/>
+    </row>
+    <row r="206" spans="2:2" s="6" customFormat="1" ht="14.5">
       <c r="B206" s="7"/>
-      <c r="C206" s="6"/>
-    </row>
-    <row r="207" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A207" s="6"/>
-      <c r="B207" s="8"/>
-      <c r="C207" s="6"/>
-    </row>
-    <row r="208" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A208" s="6"/>
-      <c r="B208" s="7"/>
-      <c r="C208" s="6"/>
-    </row>
+    </row>
+    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5">
+      <c r="B207" s="7"/>
+    </row>
+    <row r="208" spans="2:2" ht="14.25" customHeight="1"/>
     <row r="209" spans="1:3" ht="14.25" customHeight="1">
       <c r="A209" s="6"/>
-      <c r="B209" s="6"/>
+      <c r="B209" s="7"/>
       <c r="C209" s="6"/>
     </row>
     <row r="210" spans="1:3" ht="14.25" customHeight="1">
       <c r="A210" s="6"/>
-      <c r="B210" s="5"/>
+      <c r="B210" s="8"/>
       <c r="C210" s="6"/>
     </row>
     <row r="211" spans="1:3" ht="14.25" customHeight="1">
@@ -2559,12 +2620,12 @@
     </row>
     <row r="212" spans="1:3" ht="14.25" customHeight="1">
       <c r="A212" s="6"/>
-      <c r="B212" s="8"/>
+      <c r="B212" s="6"/>
       <c r="C212" s="6"/>
     </row>
     <row r="213" spans="1:3" ht="14.25" customHeight="1">
       <c r="A213" s="6"/>
-      <c r="B213" s="6"/>
+      <c r="B213" s="5"/>
       <c r="C213" s="6"/>
     </row>
     <row r="214" spans="1:3" ht="14.25" customHeight="1">
@@ -2572,23 +2633,35 @@
       <c r="B214" s="7"/>
       <c r="C214" s="6"/>
     </row>
-    <row r="215" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="215" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A215" s="6"/>
+      <c r="B215" s="8"/>
+      <c r="C215" s="6"/>
+    </row>
     <row r="216" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B216" s="5"/>
+      <c r="A216" s="6"/>
+      <c r="B216" s="6"/>
+      <c r="C216" s="6"/>
     </row>
     <row r="217" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A217" s="6"/>
       <c r="B217" s="7"/>
-    </row>
-    <row r="218" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B218" s="8"/>
-    </row>
-    <row r="219" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="C217" s="6"/>
+    </row>
+    <row r="218" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="219" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B219" s="5"/>
+    </row>
     <row r="220" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A220" s="6"/>
-    </row>
-    <row r="221" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="B220" s="7"/>
+    </row>
+    <row r="221" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B221" s="8"/>
+    </row>
     <row r="222" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="223" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="223" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A223" s="6"/>
+    </row>
     <row r="224" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="225" ht="14.25" customHeight="1"/>
     <row r="226" ht="14.25" customHeight="1"/>
@@ -3442,6 +3515,9 @@
     <row r="1074" ht="14.25" customHeight="1"/>
     <row r="1075" ht="14.25" customHeight="1"/>
     <row r="1076" ht="14.25" customHeight="1"/>
+    <row r="1077" ht="14.25" customHeight="1"/>
+    <row r="1078" ht="14.25" customHeight="1"/>
+    <row r="1079" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3636,7 +3712,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>

</xml_diff>